<commit_message>
chore: remove test row
</commit_message>
<xml_diff>
--- a/workouts/data/Workout Log.xlsx
+++ b/workouts/data/Workout Log.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="19.88" customWidth="1" style="12" min="2" max="2"/>
@@ -3641,38 +3641,6 @@
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>2099-01-01</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>Test Exercise</t>
-        </is>
-      </c>
-      <c r="D117" t="n">
-        <v>1</v>
-      </c>
-      <c r="E117" t="n">
-        <v>99</v>
-      </c>
-      <c r="F117" t="n">
-        <v>10</v>
-      </c>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>DELETE THIS ROW</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>